<commit_message>
Batch 7 reviewed and applied
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work/batch7/batch7-review.xlsx
+++ b/work/batch7/batch7-review.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maost\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\[01] Martin\[07] Claude Code\NS2-Spanish-Translation\work\batch7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{387623E7-A99F-4F26-9C3E-F5355A60E9C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC5C26A7-5586-49D8-92A7-8EFA692CCC25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{4A5C7777-D424-442B-8BC8-E09EF9913A13}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1740" uniqueCount="999">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2020" uniqueCount="999">
   <si>
     <t>Section</t>
   </si>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="B10" s="13">
         <f>COUNTA(Review!J2:J327)</f>
-        <v>46</v>
+        <v>326</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="B11" s="13">
         <f>ROWS(Review!J2:J327)-COUNTA(Review!J2:J327)</f>
-        <v>280</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="B12" s="13">
         <f>COUNTIFS(Review!G2:G327,"?*",Review!J2:J327,"")</f>
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4910,7 +4910,9 @@
       <c r="G48" s="3"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4"/>
-      <c r="J48" s="6"/>
+      <c r="J48" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K48" s="7"/>
       <c r="L48" s="7"/>
     </row>
@@ -4934,7 +4936,9 @@
       <c r="G49" s="3"/>
       <c r="H49" s="4"/>
       <c r="I49" s="4"/>
-      <c r="J49" s="6"/>
+      <c r="J49" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K49" s="7"/>
       <c r="L49" s="7"/>
     </row>
@@ -4958,7 +4962,9 @@
       <c r="G50" s="3"/>
       <c r="H50" s="4"/>
       <c r="I50" s="4"/>
-      <c r="J50" s="6"/>
+      <c r="J50" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K50" s="7"/>
       <c r="L50" s="7"/>
     </row>
@@ -4982,7 +4988,9 @@
       <c r="G51" s="3"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4"/>
-      <c r="J51" s="6"/>
+      <c r="J51" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K51" s="7"/>
       <c r="L51" s="7"/>
     </row>
@@ -5006,7 +5014,9 @@
       <c r="G52" s="3"/>
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
-      <c r="J52" s="6"/>
+      <c r="J52" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K52" s="7"/>
       <c r="L52" s="7"/>
     </row>
@@ -5030,7 +5040,9 @@
       <c r="G53" s="3"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
-      <c r="J53" s="6"/>
+      <c r="J53" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K53" s="7"/>
       <c r="L53" s="7"/>
     </row>
@@ -5054,7 +5066,9 @@
       <c r="G54" s="3"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
-      <c r="J54" s="6"/>
+      <c r="J54" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K54" s="7"/>
       <c r="L54" s="7"/>
     </row>
@@ -5078,7 +5092,9 @@
       <c r="G55" s="3"/>
       <c r="H55" s="4"/>
       <c r="I55" s="4"/>
-      <c r="J55" s="6"/>
+      <c r="J55" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K55" s="7"/>
       <c r="L55" s="7"/>
     </row>
@@ -5102,7 +5118,9 @@
       <c r="G56" s="3"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
-      <c r="J56" s="6"/>
+      <c r="J56" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K56" s="7"/>
       <c r="L56" s="7"/>
     </row>
@@ -5126,7 +5144,9 @@
       <c r="G57" s="3"/>
       <c r="H57" s="4"/>
       <c r="I57" s="4"/>
-      <c r="J57" s="6"/>
+      <c r="J57" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K57" s="7"/>
       <c r="L57" s="7"/>
     </row>
@@ -5150,7 +5170,9 @@
       <c r="G58" s="3"/>
       <c r="H58" s="4"/>
       <c r="I58" s="4"/>
-      <c r="J58" s="6"/>
+      <c r="J58" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K58" s="7"/>
       <c r="L58" s="7"/>
     </row>
@@ -5174,7 +5196,9 @@
       <c r="G59" s="3"/>
       <c r="H59" s="4"/>
       <c r="I59" s="4"/>
-      <c r="J59" s="6"/>
+      <c r="J59" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K59" s="7"/>
       <c r="L59" s="7"/>
     </row>
@@ -5198,7 +5222,9 @@
       <c r="G60" s="3"/>
       <c r="H60" s="4"/>
       <c r="I60" s="4"/>
-      <c r="J60" s="6"/>
+      <c r="J60" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K60" s="7"/>
       <c r="L60" s="7"/>
     </row>
@@ -5222,7 +5248,9 @@
       <c r="G61" s="3"/>
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
-      <c r="J61" s="6"/>
+      <c r="J61" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K61" s="7"/>
       <c r="L61" s="7"/>
     </row>
@@ -5246,7 +5274,9 @@
       <c r="G62" s="3"/>
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
-      <c r="J62" s="6"/>
+      <c r="J62" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K62" s="7"/>
       <c r="L62" s="7"/>
     </row>
@@ -5270,7 +5300,9 @@
       <c r="G63" s="3"/>
       <c r="H63" s="4"/>
       <c r="I63" s="4"/>
-      <c r="J63" s="6"/>
+      <c r="J63" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K63" s="7"/>
       <c r="L63" s="7"/>
     </row>
@@ -5294,7 +5326,9 @@
       <c r="G64" s="3"/>
       <c r="H64" s="4"/>
       <c r="I64" s="4"/>
-      <c r="J64" s="6"/>
+      <c r="J64" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K64" s="7"/>
       <c r="L64" s="7"/>
     </row>
@@ -5318,7 +5352,9 @@
       <c r="G65" s="3"/>
       <c r="H65" s="4"/>
       <c r="I65" s="4"/>
-      <c r="J65" s="6"/>
+      <c r="J65" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K65" s="7"/>
       <c r="L65" s="7"/>
     </row>
@@ -5342,7 +5378,9 @@
       <c r="G66" s="3"/>
       <c r="H66" s="4"/>
       <c r="I66" s="4"/>
-      <c r="J66" s="6"/>
+      <c r="J66" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K66" s="7"/>
       <c r="L66" s="7"/>
     </row>
@@ -5366,7 +5404,9 @@
       <c r="G67" s="3"/>
       <c r="H67" s="4"/>
       <c r="I67" s="4"/>
-      <c r="J67" s="6"/>
+      <c r="J67" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K67" s="7"/>
       <c r="L67" s="7"/>
     </row>
@@ -5394,7 +5434,9 @@
         <v>194</v>
       </c>
       <c r="I68" s="4"/>
-      <c r="J68" s="6"/>
+      <c r="J68" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K68" s="7"/>
       <c r="L68" s="7"/>
     </row>
@@ -5418,7 +5460,9 @@
       <c r="G69" s="3"/>
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
-      <c r="J69" s="6"/>
+      <c r="J69" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K69" s="7"/>
       <c r="L69" s="7"/>
     </row>
@@ -5442,7 +5486,9 @@
       <c r="G70" s="3"/>
       <c r="H70" s="4"/>
       <c r="I70" s="4"/>
-      <c r="J70" s="6"/>
+      <c r="J70" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K70" s="7"/>
       <c r="L70" s="7"/>
     </row>
@@ -5466,7 +5512,9 @@
       <c r="G71" s="3"/>
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
-      <c r="J71" s="6"/>
+      <c r="J71" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K71" s="7"/>
       <c r="L71" s="7"/>
     </row>
@@ -5490,7 +5538,9 @@
       <c r="G72" s="3"/>
       <c r="H72" s="4"/>
       <c r="I72" s="4"/>
-      <c r="J72" s="6"/>
+      <c r="J72" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K72" s="7"/>
       <c r="L72" s="7"/>
     </row>
@@ -5514,7 +5564,9 @@
       <c r="G73" s="3"/>
       <c r="H73" s="4"/>
       <c r="I73" s="4"/>
-      <c r="J73" s="6"/>
+      <c r="J73" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K73" s="7"/>
       <c r="L73" s="7"/>
     </row>
@@ -5538,7 +5590,9 @@
       <c r="G74" s="3"/>
       <c r="H74" s="4"/>
       <c r="I74" s="4"/>
-      <c r="J74" s="6"/>
+      <c r="J74" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K74" s="7"/>
       <c r="L74" s="7"/>
     </row>
@@ -5562,7 +5616,9 @@
       <c r="G75" s="3"/>
       <c r="H75" s="4"/>
       <c r="I75" s="4"/>
-      <c r="J75" s="6"/>
+      <c r="J75" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K75" s="7"/>
       <c r="L75" s="7"/>
     </row>
@@ -5586,7 +5642,9 @@
       <c r="G76" s="3"/>
       <c r="H76" s="4"/>
       <c r="I76" s="4"/>
-      <c r="J76" s="6"/>
+      <c r="J76" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K76" s="7"/>
       <c r="L76" s="7"/>
     </row>
@@ -5610,7 +5668,9 @@
       <c r="G77" s="3"/>
       <c r="H77" s="4"/>
       <c r="I77" s="4"/>
-      <c r="J77" s="6"/>
+      <c r="J77" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K77" s="7"/>
       <c r="L77" s="7"/>
     </row>
@@ -5634,7 +5694,9 @@
       <c r="G78" s="3"/>
       <c r="H78" s="4"/>
       <c r="I78" s="4"/>
-      <c r="J78" s="6"/>
+      <c r="J78" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K78" s="7"/>
       <c r="L78" s="7"/>
     </row>
@@ -5658,7 +5720,9 @@
       <c r="G79" s="3"/>
       <c r="H79" s="4"/>
       <c r="I79" s="4"/>
-      <c r="J79" s="6"/>
+      <c r="J79" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K79" s="7"/>
       <c r="L79" s="7"/>
     </row>
@@ -5682,7 +5746,9 @@
       <c r="G80" s="3"/>
       <c r="H80" s="4"/>
       <c r="I80" s="4"/>
-      <c r="J80" s="6"/>
+      <c r="J80" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K80" s="7"/>
       <c r="L80" s="7"/>
     </row>
@@ -5706,7 +5772,9 @@
       <c r="G81" s="3"/>
       <c r="H81" s="4"/>
       <c r="I81" s="4"/>
-      <c r="J81" s="6"/>
+      <c r="J81" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K81" s="7"/>
       <c r="L81" s="7"/>
     </row>
@@ -5730,7 +5798,9 @@
       <c r="G82" s="3"/>
       <c r="H82" s="4"/>
       <c r="I82" s="4"/>
-      <c r="J82" s="6"/>
+      <c r="J82" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K82" s="7"/>
       <c r="L82" s="7"/>
     </row>
@@ -5754,7 +5824,9 @@
       <c r="G83" s="3"/>
       <c r="H83" s="4"/>
       <c r="I83" s="4"/>
-      <c r="J83" s="6"/>
+      <c r="J83" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K83" s="7"/>
       <c r="L83" s="7"/>
     </row>
@@ -5778,7 +5850,9 @@
       <c r="G84" s="3"/>
       <c r="H84" s="4"/>
       <c r="I84" s="4"/>
-      <c r="J84" s="6"/>
+      <c r="J84" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K84" s="7"/>
       <c r="L84" s="7"/>
     </row>
@@ -5802,7 +5876,9 @@
       <c r="G85" s="3"/>
       <c r="H85" s="4"/>
       <c r="I85" s="4"/>
-      <c r="J85" s="6"/>
+      <c r="J85" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K85" s="7"/>
       <c r="L85" s="7"/>
     </row>
@@ -5826,7 +5902,9 @@
       <c r="G86" s="3"/>
       <c r="H86" s="4"/>
       <c r="I86" s="4"/>
-      <c r="J86" s="6"/>
+      <c r="J86" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K86" s="7"/>
       <c r="L86" s="7"/>
     </row>
@@ -5850,7 +5928,9 @@
       <c r="G87" s="3"/>
       <c r="H87" s="4"/>
       <c r="I87" s="4"/>
-      <c r="J87" s="6"/>
+      <c r="J87" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K87" s="7"/>
       <c r="L87" s="7"/>
     </row>
@@ -5874,7 +5954,9 @@
       <c r="G88" s="3"/>
       <c r="H88" s="4"/>
       <c r="I88" s="4"/>
-      <c r="J88" s="6"/>
+      <c r="J88" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K88" s="7"/>
       <c r="L88" s="7"/>
     </row>
@@ -5898,7 +5980,9 @@
       <c r="G89" s="3"/>
       <c r="H89" s="4"/>
       <c r="I89" s="4"/>
-      <c r="J89" s="6"/>
+      <c r="J89" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K89" s="7"/>
       <c r="L89" s="7"/>
     </row>
@@ -5924,7 +6008,9 @@
       <c r="I90" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="J90" s="6"/>
+      <c r="J90" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K90" s="7"/>
       <c r="L90" s="7"/>
     </row>
@@ -5950,7 +6036,9 @@
       <c r="I91" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="J91" s="6"/>
+      <c r="J91" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K91" s="7"/>
       <c r="L91" s="7"/>
     </row>
@@ -5974,7 +6062,9 @@
       <c r="G92" s="3"/>
       <c r="H92" s="4"/>
       <c r="I92" s="4"/>
-      <c r="J92" s="6"/>
+      <c r="J92" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K92" s="7"/>
       <c r="L92" s="7"/>
     </row>
@@ -5998,7 +6088,9 @@
       <c r="G93" s="3"/>
       <c r="H93" s="4"/>
       <c r="I93" s="4"/>
-      <c r="J93" s="6"/>
+      <c r="J93" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K93" s="7"/>
       <c r="L93" s="7"/>
     </row>
@@ -6022,7 +6114,9 @@
       <c r="G94" s="3"/>
       <c r="H94" s="4"/>
       <c r="I94" s="4"/>
-      <c r="J94" s="6"/>
+      <c r="J94" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K94" s="7"/>
       <c r="L94" s="7"/>
     </row>
@@ -6046,7 +6140,9 @@
       <c r="G95" s="3"/>
       <c r="H95" s="4"/>
       <c r="I95" s="4"/>
-      <c r="J95" s="6"/>
+      <c r="J95" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K95" s="7"/>
       <c r="L95" s="7"/>
     </row>
@@ -6070,7 +6166,9 @@
       <c r="G96" s="3"/>
       <c r="H96" s="4"/>
       <c r="I96" s="4"/>
-      <c r="J96" s="6"/>
+      <c r="J96" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K96" s="7"/>
       <c r="L96" s="7"/>
     </row>
@@ -6094,7 +6192,9 @@
       <c r="G97" s="3"/>
       <c r="H97" s="4"/>
       <c r="I97" s="4"/>
-      <c r="J97" s="6"/>
+      <c r="J97" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K97" s="7"/>
       <c r="L97" s="7"/>
     </row>
@@ -6118,7 +6218,9 @@
       <c r="G98" s="3"/>
       <c r="H98" s="4"/>
       <c r="I98" s="4"/>
-      <c r="J98" s="6"/>
+      <c r="J98" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K98" s="7"/>
       <c r="L98" s="7"/>
     </row>
@@ -6146,7 +6248,9 @@
         <v>284</v>
       </c>
       <c r="I99" s="4"/>
-      <c r="J99" s="6"/>
+      <c r="J99" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K99" s="7"/>
       <c r="L99" s="7"/>
     </row>
@@ -6170,7 +6274,9 @@
       <c r="G100" s="3"/>
       <c r="H100" s="4"/>
       <c r="I100" s="4"/>
-      <c r="J100" s="6"/>
+      <c r="J100" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K100" s="7"/>
       <c r="L100" s="7"/>
     </row>
@@ -6194,7 +6300,9 @@
       <c r="G101" s="3"/>
       <c r="H101" s="4"/>
       <c r="I101" s="4"/>
-      <c r="J101" s="6"/>
+      <c r="J101" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K101" s="7"/>
       <c r="L101" s="7"/>
     </row>
@@ -6220,7 +6328,9 @@
       <c r="I102" s="9" t="s">
         <v>294</v>
       </c>
-      <c r="J102" s="6"/>
+      <c r="J102" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K102" s="7"/>
       <c r="L102" s="7"/>
     </row>
@@ -6244,7 +6354,9 @@
       <c r="G103" s="3"/>
       <c r="H103" s="4"/>
       <c r="I103" s="4"/>
-      <c r="J103" s="6"/>
+      <c r="J103" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K103" s="7"/>
       <c r="L103" s="7"/>
     </row>
@@ -6268,7 +6380,9 @@
       <c r="G104" s="3"/>
       <c r="H104" s="4"/>
       <c r="I104" s="4"/>
-      <c r="J104" s="6"/>
+      <c r="J104" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K104" s="7"/>
       <c r="L104" s="7"/>
     </row>
@@ -6296,7 +6410,9 @@
         <v>304</v>
       </c>
       <c r="I105" s="4"/>
-      <c r="J105" s="6"/>
+      <c r="J105" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K105" s="7"/>
       <c r="L105" s="7"/>
     </row>
@@ -6320,7 +6436,9 @@
       <c r="G106" s="3"/>
       <c r="H106" s="4"/>
       <c r="I106" s="4"/>
-      <c r="J106" s="6"/>
+      <c r="J106" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K106" s="7"/>
       <c r="L106" s="7"/>
     </row>
@@ -6344,7 +6462,9 @@
       <c r="G107" s="3"/>
       <c r="H107" s="4"/>
       <c r="I107" s="4"/>
-      <c r="J107" s="6"/>
+      <c r="J107" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K107" s="7"/>
       <c r="L107" s="7"/>
     </row>
@@ -6368,7 +6488,9 @@
       <c r="G108" s="3"/>
       <c r="H108" s="4"/>
       <c r="I108" s="4"/>
-      <c r="J108" s="6"/>
+      <c r="J108" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K108" s="7"/>
       <c r="L108" s="7"/>
     </row>
@@ -6392,7 +6514,9 @@
       <c r="G109" s="3"/>
       <c r="H109" s="4"/>
       <c r="I109" s="4"/>
-      <c r="J109" s="6"/>
+      <c r="J109" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K109" s="7"/>
       <c r="L109" s="7"/>
     </row>
@@ -6416,7 +6540,9 @@
       <c r="G110" s="3"/>
       <c r="H110" s="4"/>
       <c r="I110" s="4"/>
-      <c r="J110" s="6"/>
+      <c r="J110" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K110" s="7"/>
       <c r="L110" s="7"/>
     </row>
@@ -6444,7 +6570,9 @@
         <v>323</v>
       </c>
       <c r="I111" s="4"/>
-      <c r="J111" s="6"/>
+      <c r="J111" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K111" s="7"/>
       <c r="L111" s="7"/>
     </row>
@@ -6468,7 +6596,9 @@
       <c r="G112" s="3"/>
       <c r="H112" s="4"/>
       <c r="I112" s="4"/>
-      <c r="J112" s="6"/>
+      <c r="J112" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K112" s="7"/>
       <c r="L112" s="7"/>
     </row>
@@ -6492,7 +6622,9 @@
       <c r="G113" s="3"/>
       <c r="H113" s="4"/>
       <c r="I113" s="4"/>
-      <c r="J113" s="6"/>
+      <c r="J113" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K113" s="7"/>
       <c r="L113" s="7"/>
     </row>
@@ -6516,7 +6648,9 @@
       <c r="G114" s="3"/>
       <c r="H114" s="4"/>
       <c r="I114" s="4"/>
-      <c r="J114" s="6"/>
+      <c r="J114" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K114" s="7"/>
       <c r="L114" s="7"/>
     </row>
@@ -6540,7 +6674,9 @@
       <c r="G115" s="3"/>
       <c r="H115" s="4"/>
       <c r="I115" s="4"/>
-      <c r="J115" s="6"/>
+      <c r="J115" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K115" s="7"/>
       <c r="L115" s="7"/>
     </row>
@@ -6564,7 +6700,9 @@
       <c r="G116" s="3"/>
       <c r="H116" s="4"/>
       <c r="I116" s="4"/>
-      <c r="J116" s="6"/>
+      <c r="J116" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K116" s="7"/>
       <c r="L116" s="7"/>
     </row>
@@ -6588,7 +6726,9 @@
       <c r="G117" s="3"/>
       <c r="H117" s="4"/>
       <c r="I117" s="4"/>
-      <c r="J117" s="6"/>
+      <c r="J117" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K117" s="7"/>
       <c r="L117" s="7"/>
     </row>
@@ -6612,7 +6752,9 @@
       <c r="G118" s="3"/>
       <c r="H118" s="4"/>
       <c r="I118" s="4"/>
-      <c r="J118" s="6"/>
+      <c r="J118" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K118" s="7"/>
       <c r="L118" s="7"/>
     </row>
@@ -6638,7 +6780,9 @@
       <c r="I119" s="9" t="s">
         <v>348</v>
       </c>
-      <c r="J119" s="6"/>
+      <c r="J119" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K119" s="7"/>
       <c r="L119" s="7"/>
     </row>
@@ -6664,7 +6808,9 @@
       <c r="I120" s="9" t="s">
         <v>352</v>
       </c>
-      <c r="J120" s="6"/>
+      <c r="J120" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K120" s="7"/>
       <c r="L120" s="7"/>
     </row>
@@ -6688,7 +6834,9 @@
       <c r="G121" s="3"/>
       <c r="H121" s="4"/>
       <c r="I121" s="4"/>
-      <c r="J121" s="6"/>
+      <c r="J121" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K121" s="7"/>
       <c r="L121" s="7"/>
     </row>
@@ -6716,7 +6864,9 @@
         <v>359</v>
       </c>
       <c r="I122" s="4"/>
-      <c r="J122" s="6"/>
+      <c r="J122" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K122" s="7"/>
       <c r="L122" s="7"/>
     </row>
@@ -6740,7 +6890,9 @@
       <c r="G123" s="3"/>
       <c r="H123" s="4"/>
       <c r="I123" s="4"/>
-      <c r="J123" s="6"/>
+      <c r="J123" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K123" s="7"/>
       <c r="L123" s="7"/>
     </row>
@@ -6764,7 +6916,9 @@
       <c r="G124" s="3"/>
       <c r="H124" s="4"/>
       <c r="I124" s="4"/>
-      <c r="J124" s="6"/>
+      <c r="J124" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K124" s="7"/>
       <c r="L124" s="7"/>
     </row>
@@ -6788,7 +6942,9 @@
       <c r="G125" s="3"/>
       <c r="H125" s="4"/>
       <c r="I125" s="4"/>
-      <c r="J125" s="6"/>
+      <c r="J125" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K125" s="7"/>
       <c r="L125" s="7"/>
     </row>
@@ -6812,7 +6968,9 @@
       <c r="G126" s="3"/>
       <c r="H126" s="4"/>
       <c r="I126" s="4"/>
-      <c r="J126" s="6"/>
+      <c r="J126" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K126" s="7"/>
       <c r="L126" s="7"/>
     </row>
@@ -6836,7 +6994,9 @@
       <c r="G127" s="3"/>
       <c r="H127" s="4"/>
       <c r="I127" s="4"/>
-      <c r="J127" s="6"/>
+      <c r="J127" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K127" s="7"/>
       <c r="L127" s="7"/>
     </row>
@@ -6860,7 +7020,9 @@
       <c r="G128" s="3"/>
       <c r="H128" s="4"/>
       <c r="I128" s="4"/>
-      <c r="J128" s="6"/>
+      <c r="J128" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K128" s="7"/>
       <c r="L128" s="7"/>
     </row>
@@ -6884,7 +7046,9 @@
       <c r="G129" s="3"/>
       <c r="H129" s="4"/>
       <c r="I129" s="4"/>
-      <c r="J129" s="6"/>
+      <c r="J129" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K129" s="7"/>
       <c r="L129" s="7"/>
     </row>
@@ -6910,7 +7074,9 @@
       <c r="I130" s="9" t="s">
         <v>384</v>
       </c>
-      <c r="J130" s="6"/>
+      <c r="J130" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K130" s="7"/>
       <c r="L130" s="7"/>
     </row>
@@ -6934,7 +7100,9 @@
       <c r="G131" s="3"/>
       <c r="H131" s="4"/>
       <c r="I131" s="4"/>
-      <c r="J131" s="6"/>
+      <c r="J131" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K131" s="7"/>
       <c r="L131" s="7"/>
     </row>
@@ -6962,7 +7130,9 @@
         <v>391</v>
       </c>
       <c r="I132" s="4"/>
-      <c r="J132" s="6"/>
+      <c r="J132" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K132" s="7"/>
       <c r="L132" s="7"/>
     </row>
@@ -6986,7 +7156,9 @@
       <c r="G133" s="3"/>
       <c r="H133" s="4"/>
       <c r="I133" s="4"/>
-      <c r="J133" s="6"/>
+      <c r="J133" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K133" s="7"/>
       <c r="L133" s="7"/>
     </row>
@@ -7010,7 +7182,9 @@
       <c r="G134" s="3"/>
       <c r="H134" s="4"/>
       <c r="I134" s="4"/>
-      <c r="J134" s="6"/>
+      <c r="J134" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K134" s="7"/>
       <c r="L134" s="7"/>
     </row>
@@ -7034,7 +7208,9 @@
       <c r="G135" s="3"/>
       <c r="H135" s="4"/>
       <c r="I135" s="4"/>
-      <c r="J135" s="6"/>
+      <c r="J135" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K135" s="7"/>
       <c r="L135" s="7"/>
     </row>
@@ -7058,7 +7234,9 @@
       <c r="G136" s="3"/>
       <c r="H136" s="4"/>
       <c r="I136" s="4"/>
-      <c r="J136" s="6"/>
+      <c r="J136" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K136" s="7"/>
       <c r="L136" s="7"/>
     </row>
@@ -7082,7 +7260,9 @@
       <c r="G137" s="3"/>
       <c r="H137" s="4"/>
       <c r="I137" s="4"/>
-      <c r="J137" s="6"/>
+      <c r="J137" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K137" s="7"/>
       <c r="L137" s="7"/>
     </row>
@@ -7106,7 +7286,9 @@
       <c r="G138" s="3"/>
       <c r="H138" s="4"/>
       <c r="I138" s="4"/>
-      <c r="J138" s="6"/>
+      <c r="J138" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K138" s="7"/>
       <c r="L138" s="7"/>
     </row>
@@ -7132,7 +7314,9 @@
       <c r="I139" s="9" t="s">
         <v>413</v>
       </c>
-      <c r="J139" s="6"/>
+      <c r="J139" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K139" s="7"/>
       <c r="L139" s="7"/>
     </row>
@@ -7156,7 +7340,9 @@
       <c r="G140" s="3"/>
       <c r="H140" s="4"/>
       <c r="I140" s="4"/>
-      <c r="J140" s="6"/>
+      <c r="J140" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K140" s="7"/>
       <c r="L140" s="7"/>
     </row>
@@ -7180,7 +7366,9 @@
       <c r="G141" s="3"/>
       <c r="H141" s="4"/>
       <c r="I141" s="4"/>
-      <c r="J141" s="6"/>
+      <c r="J141" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K141" s="7"/>
       <c r="L141" s="7"/>
     </row>
@@ -7204,7 +7392,9 @@
       <c r="G142" s="3"/>
       <c r="H142" s="4"/>
       <c r="I142" s="4"/>
-      <c r="J142" s="6"/>
+      <c r="J142" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K142" s="7"/>
       <c r="L142" s="7"/>
     </row>
@@ -7228,7 +7418,9 @@
       <c r="G143" s="3"/>
       <c r="H143" s="4"/>
       <c r="I143" s="4"/>
-      <c r="J143" s="6"/>
+      <c r="J143" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K143" s="7"/>
       <c r="L143" s="7"/>
     </row>
@@ -7252,7 +7444,9 @@
       <c r="G144" s="3"/>
       <c r="H144" s="4"/>
       <c r="I144" s="4"/>
-      <c r="J144" s="6"/>
+      <c r="J144" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K144" s="7"/>
       <c r="L144" s="7"/>
     </row>
@@ -7276,7 +7470,9 @@
       <c r="G145" s="3"/>
       <c r="H145" s="4"/>
       <c r="I145" s="4"/>
-      <c r="J145" s="6"/>
+      <c r="J145" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K145" s="7"/>
       <c r="L145" s="7"/>
     </row>
@@ -7300,7 +7496,9 @@
       <c r="G146" s="3"/>
       <c r="H146" s="4"/>
       <c r="I146" s="4"/>
-      <c r="J146" s="6"/>
+      <c r="J146" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K146" s="7"/>
       <c r="L146" s="7"/>
     </row>
@@ -7324,7 +7522,9 @@
       <c r="G147" s="3"/>
       <c r="H147" s="4"/>
       <c r="I147" s="4"/>
-      <c r="J147" s="6"/>
+      <c r="J147" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K147" s="7"/>
       <c r="L147" s="7"/>
     </row>
@@ -7348,7 +7548,9 @@
       <c r="G148" s="3"/>
       <c r="H148" s="4"/>
       <c r="I148" s="4"/>
-      <c r="J148" s="6"/>
+      <c r="J148" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K148" s="7"/>
       <c r="L148" s="7"/>
     </row>
@@ -7370,7 +7572,9 @@
       <c r="I149" s="9" t="s">
         <v>440</v>
       </c>
-      <c r="J149" s="6"/>
+      <c r="J149" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K149" s="7"/>
       <c r="L149" s="7"/>
     </row>
@@ -7394,7 +7598,9 @@
       <c r="G150" s="3"/>
       <c r="H150" s="4"/>
       <c r="I150" s="4"/>
-      <c r="J150" s="6"/>
+      <c r="J150" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K150" s="7"/>
       <c r="L150" s="7"/>
     </row>
@@ -7418,7 +7624,9 @@
       <c r="G151" s="3"/>
       <c r="H151" s="4"/>
       <c r="I151" s="4"/>
-      <c r="J151" s="6"/>
+      <c r="J151" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K151" s="7"/>
       <c r="L151" s="7"/>
     </row>
@@ -7442,7 +7650,9 @@
       <c r="G152" s="3"/>
       <c r="H152" s="4"/>
       <c r="I152" s="4"/>
-      <c r="J152" s="6"/>
+      <c r="J152" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K152" s="7"/>
       <c r="L152" s="7"/>
     </row>
@@ -7466,7 +7676,9 @@
       <c r="G153" s="3"/>
       <c r="H153" s="4"/>
       <c r="I153" s="4"/>
-      <c r="J153" s="6"/>
+      <c r="J153" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K153" s="7"/>
       <c r="L153" s="7"/>
     </row>
@@ -7490,7 +7702,9 @@
       <c r="G154" s="3"/>
       <c r="H154" s="4"/>
       <c r="I154" s="4"/>
-      <c r="J154" s="6"/>
+      <c r="J154" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K154" s="7"/>
       <c r="L154" s="7"/>
     </row>
@@ -7514,7 +7728,9 @@
       <c r="G155" s="3"/>
       <c r="H155" s="4"/>
       <c r="I155" s="4"/>
-      <c r="J155" s="6"/>
+      <c r="J155" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K155" s="7"/>
       <c r="L155" s="7"/>
     </row>
@@ -7540,7 +7756,9 @@
       <c r="I156" s="9" t="s">
         <v>462</v>
       </c>
-      <c r="J156" s="6"/>
+      <c r="J156" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K156" s="7"/>
       <c r="L156" s="7"/>
     </row>
@@ -7564,7 +7782,9 @@
       <c r="G157" s="3"/>
       <c r="H157" s="4"/>
       <c r="I157" s="4"/>
-      <c r="J157" s="6"/>
+      <c r="J157" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K157" s="7"/>
       <c r="L157" s="7"/>
     </row>
@@ -7590,7 +7810,9 @@
       <c r="I158" s="9" t="s">
         <v>294</v>
       </c>
-      <c r="J158" s="6"/>
+      <c r="J158" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K158" s="7"/>
       <c r="L158" s="7"/>
     </row>
@@ -7614,7 +7836,9 @@
       <c r="G159" s="3"/>
       <c r="H159" s="4"/>
       <c r="I159" s="4"/>
-      <c r="J159" s="6"/>
+      <c r="J159" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K159" s="7"/>
       <c r="L159" s="7"/>
     </row>
@@ -7638,7 +7862,9 @@
       <c r="G160" s="3"/>
       <c r="H160" s="4"/>
       <c r="I160" s="4"/>
-      <c r="J160" s="6"/>
+      <c r="J160" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K160" s="7"/>
       <c r="L160" s="7"/>
     </row>
@@ -7662,7 +7888,9 @@
       <c r="G161" s="3"/>
       <c r="H161" s="4"/>
       <c r="I161" s="4"/>
-      <c r="J161" s="6"/>
+      <c r="J161" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K161" s="7"/>
       <c r="L161" s="7"/>
     </row>
@@ -7686,7 +7914,9 @@
       <c r="G162" s="3"/>
       <c r="H162" s="4"/>
       <c r="I162" s="4"/>
-      <c r="J162" s="6"/>
+      <c r="J162" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K162" s="7"/>
       <c r="L162" s="7"/>
     </row>
@@ -7710,7 +7940,9 @@
       <c r="G163" s="3"/>
       <c r="H163" s="4"/>
       <c r="I163" s="4"/>
-      <c r="J163" s="6"/>
+      <c r="J163" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K163" s="7"/>
       <c r="L163" s="7"/>
     </row>
@@ -7740,7 +7972,9 @@
       <c r="I164" s="9" t="s">
         <v>482</v>
       </c>
-      <c r="J164" s="6"/>
+      <c r="J164" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K164" s="7"/>
       <c r="L164" s="7"/>
     </row>
@@ -7770,7 +8004,9 @@
       <c r="I165" s="9" t="s">
         <v>487</v>
       </c>
-      <c r="J165" s="6"/>
+      <c r="J165" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K165" s="7"/>
       <c r="L165" s="7"/>
     </row>
@@ -7794,7 +8030,9 @@
       <c r="G166" s="3"/>
       <c r="H166" s="4"/>
       <c r="I166" s="4"/>
-      <c r="J166" s="6"/>
+      <c r="J166" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K166" s="7"/>
       <c r="L166" s="7"/>
     </row>
@@ -7818,7 +8056,9 @@
       <c r="G167" s="3"/>
       <c r="H167" s="4"/>
       <c r="I167" s="4"/>
-      <c r="J167" s="6"/>
+      <c r="J167" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K167" s="7"/>
       <c r="L167" s="7"/>
     </row>
@@ -7842,7 +8082,9 @@
       <c r="G168" s="3"/>
       <c r="H168" s="4"/>
       <c r="I168" s="4"/>
-      <c r="J168" s="6"/>
+      <c r="J168" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K168" s="7"/>
       <c r="L168" s="7"/>
     </row>
@@ -7866,7 +8108,9 @@
       <c r="G169" s="3"/>
       <c r="H169" s="4"/>
       <c r="I169" s="4"/>
-      <c r="J169" s="6"/>
+      <c r="J169" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K169" s="7"/>
       <c r="L169" s="7"/>
     </row>
@@ -7892,7 +8136,9 @@
       <c r="I170" s="9" t="s">
         <v>503</v>
       </c>
-      <c r="J170" s="6"/>
+      <c r="J170" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K170" s="7"/>
       <c r="L170" s="7"/>
     </row>
@@ -7916,7 +8162,9 @@
       <c r="G171" s="3"/>
       <c r="H171" s="4"/>
       <c r="I171" s="4"/>
-      <c r="J171" s="6"/>
+      <c r="J171" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K171" s="7"/>
       <c r="L171" s="7"/>
     </row>
@@ -7940,7 +8188,9 @@
       <c r="G172" s="3"/>
       <c r="H172" s="4"/>
       <c r="I172" s="4"/>
-      <c r="J172" s="6"/>
+      <c r="J172" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K172" s="7"/>
       <c r="L172" s="7"/>
     </row>
@@ -7964,7 +8214,9 @@
       <c r="G173" s="3"/>
       <c r="H173" s="4"/>
       <c r="I173" s="4"/>
-      <c r="J173" s="6"/>
+      <c r="J173" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K173" s="7"/>
       <c r="L173" s="7"/>
     </row>
@@ -7988,7 +8240,9 @@
       <c r="G174" s="3"/>
       <c r="H174" s="4"/>
       <c r="I174" s="4"/>
-      <c r="J174" s="6"/>
+      <c r="J174" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K174" s="7"/>
       <c r="L174" s="7"/>
     </row>
@@ -8012,7 +8266,9 @@
       <c r="G175" s="3"/>
       <c r="H175" s="4"/>
       <c r="I175" s="4"/>
-      <c r="J175" s="6"/>
+      <c r="J175" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K175" s="7"/>
       <c r="L175" s="7"/>
     </row>
@@ -8036,7 +8292,9 @@
       <c r="G176" s="3"/>
       <c r="H176" s="4"/>
       <c r="I176" s="4"/>
-      <c r="J176" s="6"/>
+      <c r="J176" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K176" s="7"/>
       <c r="L176" s="7"/>
     </row>
@@ -8060,7 +8318,9 @@
       <c r="G177" s="3"/>
       <c r="H177" s="4"/>
       <c r="I177" s="4"/>
-      <c r="J177" s="6"/>
+      <c r="J177" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K177" s="7"/>
       <c r="L177" s="7"/>
     </row>
@@ -8086,7 +8346,9 @@
       <c r="I178" s="9" t="s">
         <v>528</v>
       </c>
-      <c r="J178" s="6"/>
+      <c r="J178" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K178" s="7"/>
       <c r="L178" s="7"/>
     </row>
@@ -8110,7 +8372,9 @@
       <c r="G179" s="3"/>
       <c r="H179" s="4"/>
       <c r="I179" s="4"/>
-      <c r="J179" s="6"/>
+      <c r="J179" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K179" s="7"/>
       <c r="L179" s="7"/>
     </row>
@@ -8134,7 +8398,9 @@
       <c r="G180" s="3"/>
       <c r="H180" s="4"/>
       <c r="I180" s="4"/>
-      <c r="J180" s="6"/>
+      <c r="J180" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K180" s="7"/>
       <c r="L180" s="7"/>
     </row>
@@ -8158,7 +8424,9 @@
       <c r="G181" s="3"/>
       <c r="H181" s="4"/>
       <c r="I181" s="4"/>
-      <c r="J181" s="6"/>
+      <c r="J181" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K181" s="7"/>
       <c r="L181" s="7"/>
     </row>
@@ -8182,7 +8450,9 @@
       <c r="G182" s="3"/>
       <c r="H182" s="4"/>
       <c r="I182" s="4"/>
-      <c r="J182" s="6"/>
+      <c r="J182" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K182" s="7"/>
       <c r="L182" s="7"/>
     </row>
@@ -8206,7 +8476,9 @@
       <c r="G183" s="3"/>
       <c r="H183" s="4"/>
       <c r="I183" s="4"/>
-      <c r="J183" s="6"/>
+      <c r="J183" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K183" s="7"/>
       <c r="L183" s="7"/>
     </row>
@@ -8230,7 +8502,9 @@
       <c r="G184" s="3"/>
       <c r="H184" s="4"/>
       <c r="I184" s="4"/>
-      <c r="J184" s="6"/>
+      <c r="J184" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K184" s="7"/>
       <c r="L184" s="7"/>
     </row>
@@ -8254,7 +8528,9 @@
       <c r="G185" s="3"/>
       <c r="H185" s="4"/>
       <c r="I185" s="4"/>
-      <c r="J185" s="6"/>
+      <c r="J185" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K185" s="7"/>
       <c r="L185" s="7"/>
     </row>
@@ -8278,7 +8554,9 @@
       <c r="G186" s="3"/>
       <c r="H186" s="4"/>
       <c r="I186" s="4"/>
-      <c r="J186" s="6"/>
+      <c r="J186" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K186" s="7"/>
       <c r="L186" s="7"/>
     </row>
@@ -8302,7 +8580,9 @@
       <c r="G187" s="3"/>
       <c r="H187" s="4"/>
       <c r="I187" s="4"/>
-      <c r="J187" s="6"/>
+      <c r="J187" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K187" s="7"/>
       <c r="L187" s="7"/>
     </row>
@@ -8326,7 +8606,9 @@
       <c r="G188" s="3"/>
       <c r="H188" s="4"/>
       <c r="I188" s="4"/>
-      <c r="J188" s="6"/>
+      <c r="J188" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K188" s="7"/>
       <c r="L188" s="7"/>
     </row>
@@ -8350,7 +8632,9 @@
       <c r="G189" s="3"/>
       <c r="H189" s="4"/>
       <c r="I189" s="4"/>
-      <c r="J189" s="6"/>
+      <c r="J189" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K189" s="7"/>
       <c r="L189" s="7"/>
     </row>
@@ -8374,7 +8658,9 @@
       <c r="G190" s="3"/>
       <c r="H190" s="4"/>
       <c r="I190" s="4"/>
-      <c r="J190" s="6"/>
+      <c r="J190" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K190" s="7"/>
       <c r="L190" s="7"/>
     </row>
@@ -8398,7 +8684,9 @@
       <c r="G191" s="3"/>
       <c r="H191" s="4"/>
       <c r="I191" s="4"/>
-      <c r="J191" s="6"/>
+      <c r="J191" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K191" s="7"/>
       <c r="L191" s="7"/>
     </row>
@@ -8422,7 +8710,9 @@
       <c r="G192" s="3"/>
       <c r="H192" s="4"/>
       <c r="I192" s="4"/>
-      <c r="J192" s="6"/>
+      <c r="J192" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K192" s="7"/>
       <c r="L192" s="7"/>
     </row>
@@ -8446,7 +8736,9 @@
       <c r="G193" s="3"/>
       <c r="H193" s="4"/>
       <c r="I193" s="4"/>
-      <c r="J193" s="6"/>
+      <c r="J193" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K193" s="7"/>
       <c r="L193" s="7"/>
     </row>
@@ -8470,7 +8762,9 @@
       <c r="G194" s="3"/>
       <c r="H194" s="4"/>
       <c r="I194" s="4"/>
-      <c r="J194" s="6"/>
+      <c r="J194" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K194" s="7"/>
       <c r="L194" s="7"/>
     </row>
@@ -8494,7 +8788,9 @@
       <c r="G195" s="3"/>
       <c r="H195" s="4"/>
       <c r="I195" s="4"/>
-      <c r="J195" s="6"/>
+      <c r="J195" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K195" s="7"/>
       <c r="L195" s="7"/>
     </row>
@@ -8518,7 +8814,9 @@
       <c r="G196" s="3"/>
       <c r="H196" s="4"/>
       <c r="I196" s="4"/>
-      <c r="J196" s="6"/>
+      <c r="J196" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K196" s="7"/>
       <c r="L196" s="7"/>
     </row>
@@ -8542,7 +8840,9 @@
       <c r="G197" s="3"/>
       <c r="H197" s="4"/>
       <c r="I197" s="4"/>
-      <c r="J197" s="6"/>
+      <c r="J197" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K197" s="7"/>
       <c r="L197" s="7"/>
     </row>
@@ -8566,7 +8866,9 @@
       <c r="G198" s="3"/>
       <c r="H198" s="4"/>
       <c r="I198" s="4"/>
-      <c r="J198" s="6"/>
+      <c r="J198" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K198" s="7"/>
       <c r="L198" s="7"/>
     </row>
@@ -8590,7 +8892,9 @@
       <c r="G199" s="3"/>
       <c r="H199" s="4"/>
       <c r="I199" s="4"/>
-      <c r="J199" s="6"/>
+      <c r="J199" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K199" s="7"/>
       <c r="L199" s="7"/>
     </row>
@@ -8614,7 +8918,9 @@
       <c r="G200" s="3"/>
       <c r="H200" s="4"/>
       <c r="I200" s="4"/>
-      <c r="J200" s="6"/>
+      <c r="J200" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K200" s="7"/>
       <c r="L200" s="7"/>
     </row>
@@ -8638,7 +8944,9 @@
       <c r="G201" s="3"/>
       <c r="H201" s="4"/>
       <c r="I201" s="4"/>
-      <c r="J201" s="6"/>
+      <c r="J201" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K201" s="7"/>
       <c r="L201" s="7"/>
     </row>
@@ -8662,7 +8970,9 @@
       <c r="G202" s="3"/>
       <c r="H202" s="4"/>
       <c r="I202" s="4"/>
-      <c r="J202" s="6"/>
+      <c r="J202" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K202" s="7"/>
       <c r="L202" s="7"/>
     </row>
@@ -8686,7 +8996,9 @@
       <c r="G203" s="3"/>
       <c r="H203" s="4"/>
       <c r="I203" s="4"/>
-      <c r="J203" s="6"/>
+      <c r="J203" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K203" s="7"/>
       <c r="L203" s="7"/>
     </row>
@@ -8710,7 +9022,9 @@
       <c r="G204" s="3"/>
       <c r="H204" s="4"/>
       <c r="I204" s="4"/>
-      <c r="J204" s="6"/>
+      <c r="J204" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K204" s="7"/>
       <c r="L204" s="7"/>
     </row>
@@ -8734,7 +9048,9 @@
       <c r="G205" s="3"/>
       <c r="H205" s="4"/>
       <c r="I205" s="4"/>
-      <c r="J205" s="6"/>
+      <c r="J205" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K205" s="7"/>
       <c r="L205" s="7"/>
     </row>
@@ -8758,7 +9074,9 @@
       <c r="G206" s="3"/>
       <c r="H206" s="4"/>
       <c r="I206" s="4"/>
-      <c r="J206" s="6"/>
+      <c r="J206" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K206" s="7"/>
       <c r="L206" s="7"/>
     </row>
@@ -8782,7 +9100,9 @@
       <c r="G207" s="3"/>
       <c r="H207" s="4"/>
       <c r="I207" s="4"/>
-      <c r="J207" s="6"/>
+      <c r="J207" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K207" s="7"/>
       <c r="L207" s="7"/>
     </row>
@@ -8806,7 +9126,9 @@
       <c r="G208" s="3"/>
       <c r="H208" s="4"/>
       <c r="I208" s="4"/>
-      <c r="J208" s="6"/>
+      <c r="J208" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K208" s="7"/>
       <c r="L208" s="7"/>
     </row>
@@ -8830,7 +9152,9 @@
       <c r="G209" s="3"/>
       <c r="H209" s="4"/>
       <c r="I209" s="4"/>
-      <c r="J209" s="6"/>
+      <c r="J209" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K209" s="7"/>
       <c r="L209" s="7"/>
     </row>
@@ -8854,7 +9178,9 @@
       <c r="G210" s="3"/>
       <c r="H210" s="4"/>
       <c r="I210" s="4"/>
-      <c r="J210" s="6"/>
+      <c r="J210" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K210" s="7"/>
       <c r="L210" s="7"/>
     </row>
@@ -8878,7 +9204,9 @@
       <c r="G211" s="3"/>
       <c r="H211" s="4"/>
       <c r="I211" s="4"/>
-      <c r="J211" s="6"/>
+      <c r="J211" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K211" s="7"/>
       <c r="L211" s="7"/>
     </row>
@@ -8902,7 +9230,9 @@
       <c r="G212" s="3"/>
       <c r="H212" s="4"/>
       <c r="I212" s="4"/>
-      <c r="J212" s="6"/>
+      <c r="J212" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K212" s="7"/>
       <c r="L212" s="7"/>
     </row>
@@ -8926,7 +9256,9 @@
       <c r="G213" s="3"/>
       <c r="H213" s="4"/>
       <c r="I213" s="4"/>
-      <c r="J213" s="6"/>
+      <c r="J213" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K213" s="7"/>
       <c r="L213" s="7"/>
     </row>
@@ -8950,7 +9282,9 @@
       <c r="G214" s="3"/>
       <c r="H214" s="4"/>
       <c r="I214" s="4"/>
-      <c r="J214" s="6"/>
+      <c r="J214" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K214" s="7"/>
       <c r="L214" s="7"/>
     </row>
@@ -8974,7 +9308,9 @@
       <c r="G215" s="3"/>
       <c r="H215" s="4"/>
       <c r="I215" s="4"/>
-      <c r="J215" s="6"/>
+      <c r="J215" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K215" s="7"/>
       <c r="L215" s="7"/>
     </row>
@@ -8998,7 +9334,9 @@
       <c r="G216" s="3"/>
       <c r="H216" s="4"/>
       <c r="I216" s="4"/>
-      <c r="J216" s="6"/>
+      <c r="J216" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K216" s="7"/>
       <c r="L216" s="7"/>
     </row>
@@ -9022,7 +9360,9 @@
       <c r="G217" s="3"/>
       <c r="H217" s="4"/>
       <c r="I217" s="4"/>
-      <c r="J217" s="6"/>
+      <c r="J217" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K217" s="7"/>
       <c r="L217" s="7"/>
     </row>
@@ -9046,7 +9386,9 @@
       <c r="G218" s="3"/>
       <c r="H218" s="4"/>
       <c r="I218" s="4"/>
-      <c r="J218" s="6"/>
+      <c r="J218" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K218" s="7"/>
       <c r="L218" s="7"/>
     </row>
@@ -9070,7 +9412,9 @@
       <c r="G219" s="3"/>
       <c r="H219" s="4"/>
       <c r="I219" s="4"/>
-      <c r="J219" s="6"/>
+      <c r="J219" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K219" s="7"/>
       <c r="L219" s="7"/>
     </row>
@@ -9094,7 +9438,9 @@
       <c r="G220" s="3"/>
       <c r="H220" s="4"/>
       <c r="I220" s="4"/>
-      <c r="J220" s="6"/>
+      <c r="J220" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K220" s="7"/>
       <c r="L220" s="7"/>
     </row>
@@ -9118,7 +9464,9 @@
       <c r="G221" s="3"/>
       <c r="H221" s="4"/>
       <c r="I221" s="4"/>
-      <c r="J221" s="6"/>
+      <c r="J221" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K221" s="7"/>
       <c r="L221" s="7"/>
     </row>
@@ -9142,7 +9490,9 @@
       <c r="G222" s="3"/>
       <c r="H222" s="4"/>
       <c r="I222" s="4"/>
-      <c r="J222" s="6"/>
+      <c r="J222" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K222" s="7"/>
       <c r="L222" s="7"/>
     </row>
@@ -9168,7 +9518,9 @@
         <v>664</v>
       </c>
       <c r="I223" s="4"/>
-      <c r="J223" s="6"/>
+      <c r="J223" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K223" s="7"/>
       <c r="L223" s="7"/>
     </row>
@@ -9192,7 +9544,9 @@
       <c r="G224" s="3"/>
       <c r="H224" s="4"/>
       <c r="I224" s="4"/>
-      <c r="J224" s="6"/>
+      <c r="J224" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K224" s="7"/>
       <c r="L224" s="7"/>
     </row>
@@ -9216,7 +9570,9 @@
       <c r="G225" s="3"/>
       <c r="H225" s="4"/>
       <c r="I225" s="4"/>
-      <c r="J225" s="6"/>
+      <c r="J225" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K225" s="7"/>
       <c r="L225" s="7"/>
     </row>
@@ -9240,7 +9596,9 @@
       <c r="G226" s="3"/>
       <c r="H226" s="4"/>
       <c r="I226" s="4"/>
-      <c r="J226" s="6"/>
+      <c r="J226" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K226" s="7"/>
       <c r="L226" s="7"/>
     </row>
@@ -9264,7 +9622,9 @@
       <c r="G227" s="3"/>
       <c r="H227" s="4"/>
       <c r="I227" s="4"/>
-      <c r="J227" s="6"/>
+      <c r="J227" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K227" s="7"/>
       <c r="L227" s="7"/>
     </row>
@@ -9288,7 +9648,9 @@
       <c r="G228" s="3"/>
       <c r="H228" s="4"/>
       <c r="I228" s="4"/>
-      <c r="J228" s="6"/>
+      <c r="J228" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K228" s="7"/>
       <c r="L228" s="7"/>
     </row>
@@ -9312,7 +9674,9 @@
       <c r="G229" s="3"/>
       <c r="H229" s="4"/>
       <c r="I229" s="4"/>
-      <c r="J229" s="6"/>
+      <c r="J229" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K229" s="7"/>
       <c r="L229" s="7"/>
     </row>
@@ -9336,7 +9700,9 @@
       <c r="G230" s="3"/>
       <c r="H230" s="4"/>
       <c r="I230" s="4"/>
-      <c r="J230" s="6"/>
+      <c r="J230" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K230" s="7"/>
       <c r="L230" s="7"/>
     </row>
@@ -9360,7 +9726,9 @@
       <c r="G231" s="3"/>
       <c r="H231" s="4"/>
       <c r="I231" s="4"/>
-      <c r="J231" s="6"/>
+      <c r="J231" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K231" s="7"/>
       <c r="L231" s="7"/>
     </row>
@@ -9384,7 +9752,9 @@
       <c r="G232" s="3"/>
       <c r="H232" s="4"/>
       <c r="I232" s="4"/>
-      <c r="J232" s="6"/>
+      <c r="J232" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K232" s="7"/>
       <c r="L232" s="7"/>
     </row>
@@ -9408,7 +9778,9 @@
       <c r="G233" s="3"/>
       <c r="H233" s="4"/>
       <c r="I233" s="4"/>
-      <c r="J233" s="6"/>
+      <c r="J233" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K233" s="7"/>
       <c r="L233" s="7"/>
     </row>
@@ -9432,7 +9804,9 @@
       <c r="G234" s="3"/>
       <c r="H234" s="4"/>
       <c r="I234" s="4"/>
-      <c r="J234" s="6"/>
+      <c r="J234" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K234" s="7"/>
       <c r="L234" s="7"/>
     </row>
@@ -9456,7 +9830,9 @@
       <c r="G235" s="3"/>
       <c r="H235" s="4"/>
       <c r="I235" s="4"/>
-      <c r="J235" s="6"/>
+      <c r="J235" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K235" s="7"/>
       <c r="L235" s="7"/>
     </row>
@@ -9480,7 +9856,9 @@
       <c r="G236" s="3"/>
       <c r="H236" s="4"/>
       <c r="I236" s="4"/>
-      <c r="J236" s="6"/>
+      <c r="J236" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K236" s="7"/>
       <c r="L236" s="7"/>
     </row>
@@ -9504,7 +9882,9 @@
       <c r="G237" s="3"/>
       <c r="H237" s="4"/>
       <c r="I237" s="4"/>
-      <c r="J237" s="6"/>
+      <c r="J237" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K237" s="7"/>
       <c r="L237" s="7"/>
     </row>
@@ -9528,7 +9908,9 @@
       <c r="G238" s="3"/>
       <c r="H238" s="4"/>
       <c r="I238" s="4"/>
-      <c r="J238" s="6"/>
+      <c r="J238" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K238" s="7"/>
       <c r="L238" s="7"/>
     </row>
@@ -9552,7 +9934,9 @@
       <c r="G239" s="3"/>
       <c r="H239" s="4"/>
       <c r="I239" s="4"/>
-      <c r="J239" s="6"/>
+      <c r="J239" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K239" s="7"/>
       <c r="L239" s="7"/>
     </row>
@@ -9576,7 +9960,9 @@
       <c r="G240" s="3"/>
       <c r="H240" s="4"/>
       <c r="I240" s="4"/>
-      <c r="J240" s="6"/>
+      <c r="J240" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K240" s="7"/>
       <c r="L240" s="7"/>
     </row>
@@ -9600,7 +9986,9 @@
       <c r="G241" s="3"/>
       <c r="H241" s="4"/>
       <c r="I241" s="4"/>
-      <c r="J241" s="6"/>
+      <c r="J241" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K241" s="7"/>
       <c r="L241" s="7"/>
     </row>
@@ -9624,7 +10012,9 @@
       <c r="G242" s="3"/>
       <c r="H242" s="4"/>
       <c r="I242" s="4"/>
-      <c r="J242" s="6"/>
+      <c r="J242" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K242" s="7"/>
       <c r="L242" s="7"/>
     </row>
@@ -9648,7 +10038,9 @@
       <c r="G243" s="3"/>
       <c r="H243" s="4"/>
       <c r="I243" s="4"/>
-      <c r="J243" s="6"/>
+      <c r="J243" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K243" s="7"/>
       <c r="L243" s="7"/>
     </row>
@@ -9672,7 +10064,9 @@
       <c r="G244" s="3"/>
       <c r="H244" s="4"/>
       <c r="I244" s="4"/>
-      <c r="J244" s="6"/>
+      <c r="J244" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K244" s="7"/>
       <c r="L244" s="7"/>
     </row>
@@ -9696,7 +10090,9 @@
       <c r="G245" s="3"/>
       <c r="H245" s="4"/>
       <c r="I245" s="4"/>
-      <c r="J245" s="6"/>
+      <c r="J245" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K245" s="7"/>
       <c r="L245" s="7"/>
     </row>
@@ -9720,7 +10116,9 @@
       <c r="G246" s="3"/>
       <c r="H246" s="4"/>
       <c r="I246" s="4"/>
-      <c r="J246" s="6"/>
+      <c r="J246" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K246" s="7"/>
       <c r="L246" s="7"/>
     </row>
@@ -9744,7 +10142,9 @@
       <c r="G247" s="3"/>
       <c r="H247" s="4"/>
       <c r="I247" s="4"/>
-      <c r="J247" s="6"/>
+      <c r="J247" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K247" s="7"/>
       <c r="L247" s="7"/>
     </row>
@@ -9768,7 +10168,9 @@
       <c r="G248" s="3"/>
       <c r="H248" s="4"/>
       <c r="I248" s="4"/>
-      <c r="J248" s="6"/>
+      <c r="J248" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K248" s="7"/>
       <c r="L248" s="7"/>
     </row>
@@ -9792,7 +10194,9 @@
       <c r="G249" s="3"/>
       <c r="H249" s="4"/>
       <c r="I249" s="4"/>
-      <c r="J249" s="6"/>
+      <c r="J249" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K249" s="7"/>
       <c r="L249" s="7"/>
     </row>
@@ -9816,7 +10220,9 @@
       <c r="G250" s="3"/>
       <c r="H250" s="4"/>
       <c r="I250" s="4"/>
-      <c r="J250" s="6"/>
+      <c r="J250" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K250" s="7"/>
       <c r="L250" s="7"/>
     </row>
@@ -9840,7 +10246,9 @@
       <c r="G251" s="3"/>
       <c r="H251" s="4"/>
       <c r="I251" s="4"/>
-      <c r="J251" s="6"/>
+      <c r="J251" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K251" s="7"/>
       <c r="L251" s="7"/>
     </row>
@@ -9864,7 +10272,9 @@
       <c r="G252" s="3"/>
       <c r="H252" s="4"/>
       <c r="I252" s="4"/>
-      <c r="J252" s="6"/>
+      <c r="J252" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K252" s="7"/>
       <c r="L252" s="7"/>
     </row>
@@ -9888,7 +10298,9 @@
       <c r="G253" s="3"/>
       <c r="H253" s="4"/>
       <c r="I253" s="4"/>
-      <c r="J253" s="6"/>
+      <c r="J253" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K253" s="7"/>
       <c r="L253" s="7"/>
     </row>
@@ -9912,7 +10324,9 @@
       <c r="G254" s="3"/>
       <c r="H254" s="4"/>
       <c r="I254" s="4"/>
-      <c r="J254" s="6"/>
+      <c r="J254" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K254" s="7"/>
       <c r="L254" s="7"/>
     </row>
@@ -9936,7 +10350,9 @@
       <c r="G255" s="3"/>
       <c r="H255" s="4"/>
       <c r="I255" s="4"/>
-      <c r="J255" s="6"/>
+      <c r="J255" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K255" s="7"/>
       <c r="L255" s="7"/>
     </row>
@@ -9960,7 +10376,9 @@
       <c r="G256" s="3"/>
       <c r="H256" s="4"/>
       <c r="I256" s="4"/>
-      <c r="J256" s="6"/>
+      <c r="J256" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K256" s="7"/>
       <c r="L256" s="7"/>
     </row>
@@ -9984,7 +10402,9 @@
       <c r="G257" s="3"/>
       <c r="H257" s="4"/>
       <c r="I257" s="4"/>
-      <c r="J257" s="6"/>
+      <c r="J257" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K257" s="7"/>
       <c r="L257" s="7"/>
     </row>
@@ -10008,7 +10428,9 @@
       <c r="G258" s="3"/>
       <c r="H258" s="4"/>
       <c r="I258" s="4"/>
-      <c r="J258" s="6"/>
+      <c r="J258" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K258" s="7"/>
       <c r="L258" s="7"/>
     </row>
@@ -10032,7 +10454,9 @@
       <c r="G259" s="3"/>
       <c r="H259" s="4"/>
       <c r="I259" s="4"/>
-      <c r="J259" s="6"/>
+      <c r="J259" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K259" s="7"/>
       <c r="L259" s="7"/>
     </row>
@@ -10056,7 +10480,9 @@
       <c r="G260" s="3"/>
       <c r="H260" s="4"/>
       <c r="I260" s="4"/>
-      <c r="J260" s="6"/>
+      <c r="J260" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K260" s="7"/>
       <c r="L260" s="7"/>
     </row>
@@ -10080,7 +10506,9 @@
       <c r="G261" s="3"/>
       <c r="H261" s="4"/>
       <c r="I261" s="4"/>
-      <c r="J261" s="6"/>
+      <c r="J261" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K261" s="7"/>
       <c r="L261" s="7"/>
     </row>
@@ -10104,7 +10532,9 @@
       <c r="G262" s="3"/>
       <c r="H262" s="4"/>
       <c r="I262" s="4"/>
-      <c r="J262" s="6"/>
+      <c r="J262" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K262" s="7"/>
       <c r="L262" s="7"/>
     </row>
@@ -10128,7 +10558,9 @@
       <c r="G263" s="3"/>
       <c r="H263" s="4"/>
       <c r="I263" s="4"/>
-      <c r="J263" s="6"/>
+      <c r="J263" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K263" s="7"/>
       <c r="L263" s="7"/>
     </row>
@@ -10152,7 +10584,9 @@
       <c r="G264" s="3"/>
       <c r="H264" s="4"/>
       <c r="I264" s="4"/>
-      <c r="J264" s="6"/>
+      <c r="J264" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K264" s="7"/>
       <c r="L264" s="7"/>
     </row>
@@ -10176,7 +10610,9 @@
       <c r="G265" s="3"/>
       <c r="H265" s="4"/>
       <c r="I265" s="4"/>
-      <c r="J265" s="6"/>
+      <c r="J265" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K265" s="7"/>
       <c r="L265" s="7"/>
     </row>
@@ -10200,7 +10636,9 @@
       <c r="G266" s="3"/>
       <c r="H266" s="4"/>
       <c r="I266" s="4"/>
-      <c r="J266" s="6"/>
+      <c r="J266" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K266" s="7"/>
       <c r="L266" s="7"/>
     </row>
@@ -10224,7 +10662,9 @@
       <c r="G267" s="3"/>
       <c r="H267" s="4"/>
       <c r="I267" s="4"/>
-      <c r="J267" s="6"/>
+      <c r="J267" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K267" s="7"/>
       <c r="L267" s="7"/>
     </row>
@@ -10248,7 +10688,9 @@
       <c r="G268" s="3"/>
       <c r="H268" s="4"/>
       <c r="I268" s="4"/>
-      <c r="J268" s="6"/>
+      <c r="J268" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K268" s="7"/>
       <c r="L268" s="7"/>
     </row>
@@ -10272,7 +10714,9 @@
       <c r="G269" s="3"/>
       <c r="H269" s="4"/>
       <c r="I269" s="4"/>
-      <c r="J269" s="6"/>
+      <c r="J269" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K269" s="7"/>
       <c r="L269" s="7"/>
     </row>
@@ -10296,7 +10740,9 @@
       <c r="G270" s="3"/>
       <c r="H270" s="4"/>
       <c r="I270" s="4"/>
-      <c r="J270" s="6"/>
+      <c r="J270" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K270" s="7"/>
       <c r="L270" s="7"/>
     </row>
@@ -10320,7 +10766,9 @@
       <c r="G271" s="3"/>
       <c r="H271" s="4"/>
       <c r="I271" s="4"/>
-      <c r="J271" s="6"/>
+      <c r="J271" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K271" s="7"/>
       <c r="L271" s="7"/>
     </row>
@@ -10344,7 +10792,9 @@
       <c r="G272" s="3"/>
       <c r="H272" s="4"/>
       <c r="I272" s="4"/>
-      <c r="J272" s="6"/>
+      <c r="J272" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K272" s="7"/>
       <c r="L272" s="7"/>
     </row>
@@ -10368,7 +10818,9 @@
       <c r="G273" s="3"/>
       <c r="H273" s="4"/>
       <c r="I273" s="4"/>
-      <c r="J273" s="6"/>
+      <c r="J273" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K273" s="7"/>
       <c r="L273" s="7"/>
     </row>
@@ -10392,7 +10844,9 @@
       <c r="G274" s="3"/>
       <c r="H274" s="4"/>
       <c r="I274" s="4"/>
-      <c r="J274" s="6"/>
+      <c r="J274" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K274" s="7"/>
       <c r="L274" s="7"/>
     </row>
@@ -10416,7 +10870,9 @@
       <c r="G275" s="3"/>
       <c r="H275" s="4"/>
       <c r="I275" s="4"/>
-      <c r="J275" s="6"/>
+      <c r="J275" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K275" s="7"/>
       <c r="L275" s="7"/>
     </row>
@@ -10440,7 +10896,9 @@
       <c r="G276" s="3"/>
       <c r="H276" s="4"/>
       <c r="I276" s="4"/>
-      <c r="J276" s="6"/>
+      <c r="J276" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K276" s="7"/>
       <c r="L276" s="7"/>
     </row>
@@ -10464,7 +10922,9 @@
       <c r="G277" s="3"/>
       <c r="H277" s="4"/>
       <c r="I277" s="4"/>
-      <c r="J277" s="6"/>
+      <c r="J277" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K277" s="7"/>
       <c r="L277" s="7"/>
     </row>
@@ -10488,7 +10948,9 @@
       <c r="G278" s="3"/>
       <c r="H278" s="4"/>
       <c r="I278" s="4"/>
-      <c r="J278" s="6"/>
+      <c r="J278" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K278" s="7"/>
       <c r="L278" s="7"/>
     </row>
@@ -10512,7 +10974,9 @@
       <c r="G279" s="3"/>
       <c r="H279" s="4"/>
       <c r="I279" s="4"/>
-      <c r="J279" s="6"/>
+      <c r="J279" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K279" s="7"/>
       <c r="L279" s="7"/>
     </row>
@@ -10536,7 +11000,9 @@
       <c r="G280" s="3"/>
       <c r="H280" s="4"/>
       <c r="I280" s="4"/>
-      <c r="J280" s="6"/>
+      <c r="J280" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K280" s="7"/>
       <c r="L280" s="7"/>
     </row>
@@ -10560,7 +11026,9 @@
       <c r="G281" s="3"/>
       <c r="H281" s="4"/>
       <c r="I281" s="4"/>
-      <c r="J281" s="6"/>
+      <c r="J281" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K281" s="7"/>
       <c r="L281" s="7"/>
     </row>
@@ -10584,7 +11052,9 @@
       <c r="G282" s="3"/>
       <c r="H282" s="4"/>
       <c r="I282" s="4"/>
-      <c r="J282" s="6"/>
+      <c r="J282" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K282" s="7"/>
       <c r="L282" s="7"/>
     </row>
@@ -10608,7 +11078,9 @@
       <c r="G283" s="3"/>
       <c r="H283" s="4"/>
       <c r="I283" s="4"/>
-      <c r="J283" s="6"/>
+      <c r="J283" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K283" s="7"/>
       <c r="L283" s="7"/>
     </row>
@@ -10632,7 +11104,9 @@
       <c r="G284" s="3"/>
       <c r="H284" s="4"/>
       <c r="I284" s="4"/>
-      <c r="J284" s="6"/>
+      <c r="J284" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K284" s="7"/>
       <c r="L284" s="7"/>
     </row>
@@ -10658,7 +11132,9 @@
       <c r="I285" s="9" t="s">
         <v>384</v>
       </c>
-      <c r="J285" s="6"/>
+      <c r="J285" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K285" s="7"/>
       <c r="L285" s="7"/>
     </row>
@@ -10682,7 +11158,9 @@
       <c r="G286" s="3"/>
       <c r="H286" s="4"/>
       <c r="I286" s="4"/>
-      <c r="J286" s="6"/>
+      <c r="J286" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K286" s="7"/>
       <c r="L286" s="7"/>
     </row>
@@ -10706,7 +11184,9 @@
       <c r="G287" s="3"/>
       <c r="H287" s="4"/>
       <c r="I287" s="4"/>
-      <c r="J287" s="6"/>
+      <c r="J287" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K287" s="7"/>
       <c r="L287" s="7"/>
     </row>
@@ -10730,7 +11210,9 @@
       <c r="G288" s="3"/>
       <c r="H288" s="4"/>
       <c r="I288" s="4"/>
-      <c r="J288" s="6"/>
+      <c r="J288" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K288" s="7"/>
       <c r="L288" s="7"/>
     </row>
@@ -10754,7 +11236,9 @@
       <c r="G289" s="3"/>
       <c r="H289" s="4"/>
       <c r="I289" s="4"/>
-      <c r="J289" s="6"/>
+      <c r="J289" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K289" s="7"/>
       <c r="L289" s="7"/>
     </row>
@@ -10778,7 +11262,9 @@
       <c r="G290" s="3"/>
       <c r="H290" s="4"/>
       <c r="I290" s="4"/>
-      <c r="J290" s="6"/>
+      <c r="J290" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K290" s="7"/>
       <c r="L290" s="7"/>
     </row>
@@ -10802,7 +11288,9 @@
       <c r="G291" s="3"/>
       <c r="H291" s="4"/>
       <c r="I291" s="4"/>
-      <c r="J291" s="6"/>
+      <c r="J291" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K291" s="7"/>
       <c r="L291" s="7"/>
     </row>
@@ -10826,7 +11314,9 @@
       <c r="G292" s="3"/>
       <c r="H292" s="4"/>
       <c r="I292" s="4"/>
-      <c r="J292" s="6"/>
+      <c r="J292" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K292" s="7"/>
       <c r="L292" s="7"/>
     </row>
@@ -10850,7 +11340,9 @@
       <c r="G293" s="3"/>
       <c r="H293" s="4"/>
       <c r="I293" s="4"/>
-      <c r="J293" s="6"/>
+      <c r="J293" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K293" s="7"/>
       <c r="L293" s="7"/>
     </row>
@@ -10874,7 +11366,9 @@
       <c r="G294" s="3"/>
       <c r="H294" s="4"/>
       <c r="I294" s="4"/>
-      <c r="J294" s="6"/>
+      <c r="J294" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K294" s="7"/>
       <c r="L294" s="7"/>
     </row>
@@ -10898,7 +11392,9 @@
       <c r="G295" s="3"/>
       <c r="H295" s="4"/>
       <c r="I295" s="4"/>
-      <c r="J295" s="6"/>
+      <c r="J295" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K295" s="7"/>
       <c r="L295" s="7"/>
     </row>
@@ -10922,7 +11418,9 @@
       <c r="G296" s="3"/>
       <c r="H296" s="4"/>
       <c r="I296" s="4"/>
-      <c r="J296" s="6"/>
+      <c r="J296" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K296" s="7"/>
       <c r="L296" s="7"/>
     </row>
@@ -10946,7 +11444,9 @@
       <c r="G297" s="3"/>
       <c r="H297" s="4"/>
       <c r="I297" s="4"/>
-      <c r="J297" s="6"/>
+      <c r="J297" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K297" s="7"/>
       <c r="L297" s="7"/>
     </row>
@@ -10970,7 +11470,9 @@
       <c r="G298" s="3"/>
       <c r="H298" s="4"/>
       <c r="I298" s="4"/>
-      <c r="J298" s="6"/>
+      <c r="J298" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K298" s="7"/>
       <c r="L298" s="7"/>
     </row>
@@ -10994,7 +11496,9 @@
       <c r="G299" s="3"/>
       <c r="H299" s="4"/>
       <c r="I299" s="4"/>
-      <c r="J299" s="6"/>
+      <c r="J299" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K299" s="7"/>
       <c r="L299" s="7"/>
     </row>
@@ -11018,7 +11522,9 @@
       <c r="G300" s="3"/>
       <c r="H300" s="4"/>
       <c r="I300" s="4"/>
-      <c r="J300" s="6"/>
+      <c r="J300" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K300" s="7"/>
       <c r="L300" s="7"/>
     </row>
@@ -11042,7 +11548,9 @@
       <c r="G301" s="3"/>
       <c r="H301" s="4"/>
       <c r="I301" s="4"/>
-      <c r="J301" s="6"/>
+      <c r="J301" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K301" s="7"/>
       <c r="L301" s="7"/>
     </row>
@@ -11066,7 +11574,9 @@
       <c r="G302" s="3"/>
       <c r="H302" s="4"/>
       <c r="I302" s="4"/>
-      <c r="J302" s="6"/>
+      <c r="J302" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K302" s="7"/>
       <c r="L302" s="7"/>
     </row>
@@ -11090,7 +11600,9 @@
       <c r="G303" s="3"/>
       <c r="H303" s="4"/>
       <c r="I303" s="4"/>
-      <c r="J303" s="6"/>
+      <c r="J303" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K303" s="7"/>
       <c r="L303" s="7"/>
     </row>
@@ -11114,7 +11626,9 @@
       <c r="G304" s="3"/>
       <c r="H304" s="4"/>
       <c r="I304" s="4"/>
-      <c r="J304" s="6"/>
+      <c r="J304" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K304" s="7"/>
       <c r="L304" s="7"/>
     </row>
@@ -11140,7 +11654,9 @@
       <c r="I305" s="9" t="s">
         <v>909</v>
       </c>
-      <c r="J305" s="6"/>
+      <c r="J305" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K305" s="7"/>
       <c r="L305" s="7"/>
     </row>
@@ -11164,7 +11680,9 @@
       <c r="G306" s="3"/>
       <c r="H306" s="4"/>
       <c r="I306" s="4"/>
-      <c r="J306" s="6"/>
+      <c r="J306" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K306" s="7"/>
       <c r="L306" s="7"/>
     </row>
@@ -11188,7 +11706,9 @@
       <c r="G307" s="3"/>
       <c r="H307" s="4"/>
       <c r="I307" s="4"/>
-      <c r="J307" s="6"/>
+      <c r="J307" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K307" s="7"/>
       <c r="L307" s="7"/>
     </row>
@@ -11212,7 +11732,9 @@
       <c r="G308" s="3"/>
       <c r="H308" s="4"/>
       <c r="I308" s="4"/>
-      <c r="J308" s="6"/>
+      <c r="J308" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K308" s="7"/>
       <c r="L308" s="7"/>
     </row>
@@ -11236,7 +11758,9 @@
       <c r="G309" s="3"/>
       <c r="H309" s="4"/>
       <c r="I309" s="4"/>
-      <c r="J309" s="6"/>
+      <c r="J309" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K309" s="7"/>
       <c r="L309" s="7"/>
     </row>
@@ -11260,7 +11784,9 @@
       <c r="G310" s="3"/>
       <c r="H310" s="4"/>
       <c r="I310" s="4"/>
-      <c r="J310" s="6"/>
+      <c r="J310" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K310" s="7"/>
       <c r="L310" s="7"/>
     </row>
@@ -11284,7 +11810,9 @@
       <c r="G311" s="3"/>
       <c r="H311" s="4"/>
       <c r="I311" s="4"/>
-      <c r="J311" s="6"/>
+      <c r="J311" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K311" s="7"/>
       <c r="L311" s="7"/>
     </row>
@@ -11308,7 +11836,9 @@
       <c r="G312" s="3"/>
       <c r="H312" s="4"/>
       <c r="I312" s="4"/>
-      <c r="J312" s="6"/>
+      <c r="J312" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K312" s="7"/>
       <c r="L312" s="7"/>
     </row>
@@ -11332,7 +11862,9 @@
       <c r="G313" s="3"/>
       <c r="H313" s="4"/>
       <c r="I313" s="4"/>
-      <c r="J313" s="6"/>
+      <c r="J313" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K313" s="7"/>
       <c r="L313" s="7"/>
     </row>
@@ -11356,7 +11888,9 @@
       <c r="G314" s="3"/>
       <c r="H314" s="4"/>
       <c r="I314" s="4"/>
-      <c r="J314" s="6"/>
+      <c r="J314" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K314" s="7"/>
       <c r="L314" s="7"/>
     </row>
@@ -11380,7 +11914,9 @@
       <c r="G315" s="3"/>
       <c r="H315" s="4"/>
       <c r="I315" s="4"/>
-      <c r="J315" s="6"/>
+      <c r="J315" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K315" s="7"/>
       <c r="L315" s="7"/>
     </row>
@@ -11404,7 +11940,9 @@
       <c r="G316" s="3"/>
       <c r="H316" s="4"/>
       <c r="I316" s="4"/>
-      <c r="J316" s="6"/>
+      <c r="J316" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K316" s="7"/>
       <c r="L316" s="7"/>
     </row>
@@ -11428,7 +11966,9 @@
       <c r="G317" s="3"/>
       <c r="H317" s="4"/>
       <c r="I317" s="4"/>
-      <c r="J317" s="6"/>
+      <c r="J317" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K317" s="7"/>
       <c r="L317" s="7"/>
     </row>
@@ -11452,7 +11992,9 @@
       <c r="G318" s="3"/>
       <c r="H318" s="4"/>
       <c r="I318" s="4"/>
-      <c r="J318" s="6"/>
+      <c r="J318" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K318" s="7"/>
       <c r="L318" s="7"/>
     </row>
@@ -11476,7 +12018,9 @@
       <c r="G319" s="3"/>
       <c r="H319" s="4"/>
       <c r="I319" s="4"/>
-      <c r="J319" s="6"/>
+      <c r="J319" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K319" s="7"/>
       <c r="L319" s="7"/>
     </row>
@@ -11500,7 +12044,9 @@
       <c r="G320" s="3"/>
       <c r="H320" s="4"/>
       <c r="I320" s="4"/>
-      <c r="J320" s="6"/>
+      <c r="J320" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K320" s="7"/>
       <c r="L320" s="7"/>
     </row>
@@ -11524,7 +12070,9 @@
       <c r="G321" s="3"/>
       <c r="H321" s="4"/>
       <c r="I321" s="4"/>
-      <c r="J321" s="6"/>
+      <c r="J321" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K321" s="7"/>
       <c r="L321" s="7"/>
     </row>
@@ -11548,7 +12096,9 @@
       <c r="G322" s="3"/>
       <c r="H322" s="4"/>
       <c r="I322" s="4"/>
-      <c r="J322" s="6"/>
+      <c r="J322" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K322" s="7"/>
       <c r="L322" s="7"/>
     </row>
@@ -11572,7 +12122,9 @@
       <c r="G323" s="3"/>
       <c r="H323" s="4"/>
       <c r="I323" s="4"/>
-      <c r="J323" s="6"/>
+      <c r="J323" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K323" s="7"/>
       <c r="L323" s="7"/>
     </row>
@@ -11596,7 +12148,9 @@
       <c r="G324" s="3"/>
       <c r="H324" s="4"/>
       <c r="I324" s="4"/>
-      <c r="J324" s="6"/>
+      <c r="J324" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K324" s="7"/>
       <c r="L324" s="7"/>
     </row>
@@ -11620,7 +12174,9 @@
       <c r="G325" s="3"/>
       <c r="H325" s="4"/>
       <c r="I325" s="4"/>
-      <c r="J325" s="6"/>
+      <c r="J325" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K325" s="7"/>
       <c r="L325" s="7"/>
     </row>
@@ -11644,7 +12200,9 @@
       <c r="G326" s="3"/>
       <c r="H326" s="4"/>
       <c r="I326" s="4"/>
-      <c r="J326" s="6"/>
+      <c r="J326" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K326" s="7"/>
       <c r="L326" s="7"/>
     </row>
@@ -11668,7 +12226,9 @@
       <c r="G327" s="3"/>
       <c r="H327" s="4"/>
       <c r="I327" s="4"/>
-      <c r="J327" s="6"/>
+      <c r="J327" s="6" t="s">
+        <v>984</v>
+      </c>
       <c r="K327" s="7"/>
       <c r="L327" s="7"/>
     </row>

</xml_diff>